<commit_message>
özellik: kademe aralığı olan taslağa geçildi
</commit_message>
<xml_diff>
--- a/docs/cikti_taslagi.xlsx
+++ b/docs/cikti_taslagi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammed.bulut\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D19E49E-CD3E-4BD6-85E5-BF551FF9C91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641C9AEA-0D55-4354-B71B-FE0CF98FAFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
     <definedName name="ilanNo">#REF!</definedName>
     <definedName name="MTarihi">#REF!</definedName>
     <definedName name="Muhammed_Taha_Kayaoğlu">[1]AG!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Karar Tutanağı'!$B$2:$L$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Karar Tutanağı'!$B$2:$L$32</definedName>
     <definedName name="YIL">[2]Adaylar!$CE$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">AD SOYAD </t>
   </si>
@@ -125,7 +125,13 @@
     <t>BRÜT ÜCRET (TL)</t>
   </si>
   <si>
-    <t>Toplam</t>
+    <t>Toplam Prim Gün Sayısı</t>
+  </si>
+  <si>
+    <t>Yıl Gün Ay</t>
+  </si>
+  <si>
+    <t>DK Aralığı</t>
   </si>
 </sst>
 </file>
@@ -433,7 +439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -462,12 +468,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -550,189 +550,125 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Virgül 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="153">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="144">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2510,7 +2446,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AM31"/>
+  <dimension ref="B1:AM32"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.44140625" customWidth="1"/>
@@ -2530,31 +2466,31 @@
   <sheetData>
     <row r="1" spans="2:39" s="1" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:39" s="1" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="F2" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="34" t="s">
+      <c r="G2" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="48" t="s">
+      <c r="H2" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="50"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="55"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
@@ -2569,17 +2505,17 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" spans="2:39" s="1" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="53"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="58"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -2594,19 +2530,19 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="2:39" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="60"/>
+      <c r="I4" s="60"/>
+      <c r="J4" s="60"/>
+      <c r="K4" s="60"/>
+      <c r="L4" s="60"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -2624,25 +2560,25 @@
       <c r="AC4" s="2"/>
     </row>
     <row r="5" spans="2:39" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="17"/>
-      <c r="C5" s="39" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39" t="s">
+      <c r="D5" s="60"/>
+      <c r="E5" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39" t="s">
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="J5" s="39"/>
-      <c r="K5" s="39" t="s">
+      <c r="J5" s="60"/>
+      <c r="K5" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="39"/>
+      <c r="L5" s="60"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -2660,161 +2596,161 @@
       <c r="AC5" s="2"/>
     </row>
     <row r="6" spans="2:39" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="20"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="55"/>
-      <c r="J6" s="55"/>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
-      <c r="S6" s="13"/>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="X6" s="13"/>
-      <c r="Y6" s="13"/>
-      <c r="Z6" s="13"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="61"/>
+      <c r="J6" s="61"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="11"/>
+      <c r="R6" s="11"/>
+      <c r="S6" s="11"/>
+      <c r="T6" s="11"/>
+      <c r="U6" s="11"/>
+      <c r="V6" s="11"/>
+      <c r="W6" s="11"/>
+      <c r="X6" s="11"/>
+      <c r="Y6" s="11"/>
+      <c r="Z6" s="11"/>
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="2"/>
     </row>
     <row r="7" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="20"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="40"/>
-      <c r="L7" s="40"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="13"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
-      <c r="W7" s="13"/>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="13"/>
-      <c r="Z7" s="13"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="51"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="49"/>
+      <c r="L7" s="49"/>
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="11"/>
+      <c r="S7" s="11"/>
+      <c r="T7" s="11"/>
+      <c r="U7" s="11"/>
+      <c r="V7" s="11"/>
+      <c r="W7" s="11"/>
+      <c r="X7" s="11"/>
+      <c r="Y7" s="11"/>
+      <c r="Z7" s="11"/>
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
     </row>
     <row r="8" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="20"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="56"/>
-      <c r="L8" s="56"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="13"/>
-      <c r="R8" s="13"/>
-      <c r="S8" s="13"/>
-      <c r="T8" s="13"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="13"/>
-      <c r="W8" s="13"/>
-      <c r="X8" s="13"/>
-      <c r="Y8" s="13"/>
-      <c r="Z8" s="13"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="51"/>
+      <c r="J8" s="52"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
+      <c r="S8" s="11"/>
+      <c r="T8" s="11"/>
+      <c r="U8" s="11"/>
+      <c r="V8" s="11"/>
+      <c r="W8" s="11"/>
+      <c r="X8" s="11"/>
+      <c r="Y8" s="11"/>
+      <c r="Z8" s="11"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
     </row>
     <row r="9" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="20"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="43"/>
-      <c r="K9" s="56"/>
-      <c r="L9" s="56"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="13"/>
-      <c r="S9" s="13"/>
-      <c r="T9" s="13"/>
-      <c r="U9" s="13"/>
-      <c r="V9" s="13"/>
-      <c r="W9" s="13"/>
-      <c r="X9" s="13"/>
-      <c r="Y9" s="13"/>
-      <c r="Z9" s="13"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="52"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="48"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11"/>
+      <c r="T9" s="11"/>
+      <c r="U9" s="11"/>
+      <c r="V9" s="11"/>
+      <c r="W9" s="11"/>
+      <c r="X9" s="11"/>
+      <c r="Y9" s="11"/>
+      <c r="Z9" s="11"/>
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
     </row>
     <row r="10" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="20"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="43"/>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
-      <c r="R10" s="13"/>
-      <c r="S10" s="13"/>
-      <c r="T10" s="13"/>
-      <c r="U10" s="13"/>
-      <c r="V10" s="13"/>
-      <c r="W10" s="13"/>
-      <c r="X10" s="13"/>
-      <c r="Y10" s="13"/>
-      <c r="Z10" s="13"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="52"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11"/>
+      <c r="T10" s="11"/>
+      <c r="U10" s="11"/>
+      <c r="V10" s="11"/>
+      <c r="W10" s="11"/>
+      <c r="X10" s="11"/>
+      <c r="Y10" s="11"/>
+      <c r="Z10" s="11"/>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
     </row>
     <row r="11" spans="2:39" s="1" customFormat="1" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39" t="s">
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39"/>
-      <c r="J11" s="39"/>
-      <c r="K11" s="39"/>
-      <c r="L11" s="39"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="60"/>
+      <c r="L11" s="60"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
@@ -2832,47 +2768,47 @@
       <c r="AC11" s="2"/>
     </row>
     <row r="12" spans="2:39" s="1" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="21" t="s">
+      <c r="E12" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="47" t="s">
+      <c r="G12" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
-      <c r="J12" s="14" t="s">
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
+      <c r="J12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="K12" s="14" t="s">
+      <c r="K12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="L12" s="14" t="s">
+      <c r="L12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="O12" s="54"/>
-      <c r="P12" s="54"/>
-      <c r="Q12" s="54"/>
-      <c r="R12" s="37"/>
+      <c r="O12" s="59"/>
+      <c r="P12" s="59"/>
+      <c r="Q12" s="59"/>
+      <c r="R12" s="35"/>
       <c r="S12" s="5"/>
-      <c r="T12" s="54"/>
-      <c r="U12" s="54"/>
-      <c r="V12" s="54"/>
+      <c r="T12" s="59"/>
+      <c r="U12" s="59"/>
+      <c r="V12" s="59"/>
       <c r="W12" s="5"/>
-      <c r="X12" s="54"/>
-      <c r="Y12" s="54"/>
-      <c r="Z12" s="54"/>
+      <c r="X12" s="59"/>
+      <c r="Y12" s="59"/>
+      <c r="Z12" s="59"/>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
@@ -2887,590 +2823,590 @@
       <c r="AL12" s="4"/>
       <c r="AM12" s="4"/>
     </row>
-    <row r="13" spans="2:39" s="29" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="23"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="57"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="38"/>
-      <c r="O13" s="28"/>
-      <c r="P13" s="28"/>
-      <c r="Q13" s="28"/>
-      <c r="R13" s="28"/>
+    <row r="13" spans="2:39" s="27" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="47"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="24"/>
+      <c r="L13" s="36"/>
+      <c r="O13" s="26"/>
+      <c r="P13" s="26"/>
+      <c r="Q13" s="26"/>
+      <c r="R13" s="26"/>
       <c r="S13" s="5"/>
-      <c r="T13" s="28"/>
-      <c r="U13" s="28"/>
-      <c r="V13" s="28"/>
+      <c r="T13" s="26"/>
+      <c r="U13" s="26"/>
+      <c r="V13" s="26"/>
       <c r="W13" s="5"/>
-      <c r="X13" s="28"/>
-      <c r="Y13" s="28"/>
-      <c r="Z13" s="28"/>
-      <c r="AA13" s="30"/>
-      <c r="AB13" s="30"/>
-      <c r="AC13" s="30"/>
-      <c r="AD13" s="31"/>
-      <c r="AE13" s="31"/>
-      <c r="AF13" s="31"/>
-      <c r="AG13" s="31"/>
-      <c r="AH13" s="31"/>
-      <c r="AI13" s="31"/>
-      <c r="AJ13" s="31"/>
-      <c r="AK13" s="31"/>
-      <c r="AL13" s="31"/>
-      <c r="AM13" s="31"/>
+      <c r="X13" s="26"/>
+      <c r="Y13" s="26"/>
+      <c r="Z13" s="26"/>
+      <c r="AA13" s="28"/>
+      <c r="AB13" s="28"/>
+      <c r="AC13" s="28"/>
+      <c r="AD13" s="29"/>
+      <c r="AE13" s="29"/>
+      <c r="AF13" s="29"/>
+      <c r="AG13" s="29"/>
+      <c r="AH13" s="29"/>
+      <c r="AI13" s="29"/>
+      <c r="AJ13" s="29"/>
+      <c r="AK13" s="29"/>
+      <c r="AL13" s="29"/>
+      <c r="AM13" s="29"/>
     </row>
-    <row r="14" spans="2:39" s="29" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="23"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="58"/>
-      <c r="I14" s="59"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="38"/>
-      <c r="O14" s="28"/>
-      <c r="P14" s="28"/>
-      <c r="Q14" s="28"/>
-      <c r="R14" s="28"/>
+    <row r="14" spans="2:39" s="27" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="36"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="26"/>
+      <c r="Q14" s="26"/>
+      <c r="R14" s="26"/>
       <c r="S14" s="5"/>
-      <c r="T14" s="28"/>
-      <c r="U14" s="28"/>
-      <c r="V14" s="28"/>
+      <c r="T14" s="26"/>
+      <c r="U14" s="26"/>
+      <c r="V14" s="26"/>
       <c r="W14" s="5"/>
-      <c r="X14" s="28"/>
-      <c r="Y14" s="28"/>
-      <c r="Z14" s="28"/>
-      <c r="AA14" s="30"/>
-      <c r="AB14" s="30"/>
-      <c r="AC14" s="30"/>
-      <c r="AD14" s="31"/>
-      <c r="AE14" s="31"/>
-      <c r="AF14" s="31"/>
-      <c r="AG14" s="31"/>
-      <c r="AH14" s="31"/>
-      <c r="AI14" s="31"/>
-      <c r="AJ14" s="31"/>
-      <c r="AK14" s="31"/>
-      <c r="AL14" s="31"/>
-      <c r="AM14" s="31"/>
+      <c r="X14" s="26"/>
+      <c r="Y14" s="26"/>
+      <c r="Z14" s="26"/>
+      <c r="AA14" s="28"/>
+      <c r="AB14" s="28"/>
+      <c r="AC14" s="28"/>
+      <c r="AD14" s="29"/>
+      <c r="AE14" s="29"/>
+      <c r="AF14" s="29"/>
+      <c r="AG14" s="29"/>
+      <c r="AH14" s="29"/>
+      <c r="AI14" s="29"/>
+      <c r="AJ14" s="29"/>
+      <c r="AK14" s="29"/>
+      <c r="AL14" s="29"/>
+      <c r="AM14" s="29"/>
     </row>
-    <row r="15" spans="2:39" s="29" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="23"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="57"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="59"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="38"/>
-      <c r="O15" s="28"/>
-      <c r="P15" s="28"/>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="28"/>
+    <row r="15" spans="2:39" s="27" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="36"/>
+      <c r="O15" s="26"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="26"/>
+      <c r="R15" s="26"/>
       <c r="S15" s="5"/>
-      <c r="T15" s="28"/>
-      <c r="U15" s="28"/>
-      <c r="V15" s="28"/>
+      <c r="T15" s="26"/>
+      <c r="U15" s="26"/>
+      <c r="V15" s="26"/>
       <c r="W15" s="5"/>
-      <c r="X15" s="28"/>
-      <c r="Y15" s="28"/>
-      <c r="Z15" s="28"/>
-      <c r="AA15" s="30"/>
-      <c r="AB15" s="30"/>
-      <c r="AC15" s="30"/>
-      <c r="AD15" s="31"/>
-      <c r="AE15" s="31"/>
-      <c r="AF15" s="31"/>
-      <c r="AG15" s="31"/>
-      <c r="AH15" s="31"/>
-      <c r="AI15" s="31"/>
-      <c r="AJ15" s="31"/>
-      <c r="AK15" s="31"/>
-      <c r="AL15" s="31"/>
-      <c r="AM15" s="31"/>
+      <c r="X15" s="26"/>
+      <c r="Y15" s="26"/>
+      <c r="Z15" s="26"/>
+      <c r="AA15" s="28"/>
+      <c r="AB15" s="28"/>
+      <c r="AC15" s="28"/>
+      <c r="AD15" s="29"/>
+      <c r="AE15" s="29"/>
+      <c r="AF15" s="29"/>
+      <c r="AG15" s="29"/>
+      <c r="AH15" s="29"/>
+      <c r="AI15" s="29"/>
+      <c r="AJ15" s="29"/>
+      <c r="AK15" s="29"/>
+      <c r="AL15" s="29"/>
+      <c r="AM15" s="29"/>
     </row>
-    <row r="16" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="23"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="57"/>
-      <c r="H16" s="58"/>
-      <c r="I16" s="59"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="38"/>
-      <c r="O16" s="27"/>
-      <c r="P16" s="27"/>
-      <c r="Q16" s="27"/>
-      <c r="R16" s="27"/>
+    <row r="16" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="47"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="36"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="25"/>
+      <c r="R16" s="25"/>
       <c r="S16" s="5"/>
-      <c r="T16" s="27"/>
-      <c r="U16" s="27"/>
-      <c r="V16" s="27"/>
+      <c r="T16" s="25"/>
+      <c r="U16" s="25"/>
+      <c r="V16" s="25"/>
       <c r="W16" s="5"/>
-      <c r="X16" s="27"/>
-      <c r="Y16" s="27"/>
-      <c r="Z16" s="27"/>
-      <c r="AA16" s="30"/>
-      <c r="AB16" s="30"/>
-      <c r="AC16" s="30"/>
-      <c r="AD16" s="31"/>
-      <c r="AE16" s="31"/>
-      <c r="AF16" s="31"/>
-      <c r="AG16" s="31"/>
-      <c r="AH16" s="31"/>
-      <c r="AI16" s="31"/>
-      <c r="AJ16" s="31"/>
-      <c r="AK16" s="31"/>
-      <c r="AL16" s="31"/>
-      <c r="AM16" s="31"/>
+      <c r="X16" s="25"/>
+      <c r="Y16" s="25"/>
+      <c r="Z16" s="25"/>
+      <c r="AA16" s="28"/>
+      <c r="AB16" s="28"/>
+      <c r="AC16" s="28"/>
+      <c r="AD16" s="29"/>
+      <c r="AE16" s="29"/>
+      <c r="AF16" s="29"/>
+      <c r="AG16" s="29"/>
+      <c r="AH16" s="29"/>
+      <c r="AI16" s="29"/>
+      <c r="AJ16" s="29"/>
+      <c r="AK16" s="29"/>
+      <c r="AL16" s="29"/>
+      <c r="AM16" s="29"/>
     </row>
-    <row r="17" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="58"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="38"/>
-      <c r="O17" s="32"/>
-      <c r="P17" s="32"/>
-      <c r="Q17" s="32"/>
-      <c r="R17" s="32"/>
+    <row r="17" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="21"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="47"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="36"/>
+      <c r="O17" s="30"/>
+      <c r="P17" s="30"/>
+      <c r="Q17" s="30"/>
+      <c r="R17" s="30"/>
       <c r="S17" s="5"/>
-      <c r="T17" s="32"/>
-      <c r="U17" s="32"/>
-      <c r="V17" s="32"/>
+      <c r="T17" s="30"/>
+      <c r="U17" s="30"/>
+      <c r="V17" s="30"/>
       <c r="W17" s="5"/>
-      <c r="X17" s="32"/>
-      <c r="Y17" s="32"/>
-      <c r="Z17" s="32"/>
-      <c r="AA17" s="30"/>
-      <c r="AB17" s="30"/>
-      <c r="AC17" s="30"/>
-      <c r="AD17" s="31"/>
-      <c r="AE17" s="31"/>
-      <c r="AF17" s="31"/>
-      <c r="AG17" s="31"/>
-      <c r="AH17" s="31"/>
-      <c r="AI17" s="31"/>
-      <c r="AJ17" s="31"/>
-      <c r="AK17" s="31"/>
-      <c r="AL17" s="31"/>
-      <c r="AM17" s="31"/>
+      <c r="X17" s="30"/>
+      <c r="Y17" s="30"/>
+      <c r="Z17" s="30"/>
+      <c r="AA17" s="28"/>
+      <c r="AB17" s="28"/>
+      <c r="AC17" s="28"/>
+      <c r="AD17" s="29"/>
+      <c r="AE17" s="29"/>
+      <c r="AF17" s="29"/>
+      <c r="AG17" s="29"/>
+      <c r="AH17" s="29"/>
+      <c r="AI17" s="29"/>
+      <c r="AJ17" s="29"/>
+      <c r="AK17" s="29"/>
+      <c r="AL17" s="29"/>
+      <c r="AM17" s="29"/>
     </row>
-    <row r="18" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="23"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="57"/>
-      <c r="H18" s="58"/>
-      <c r="I18" s="59"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="38"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="37"/>
-      <c r="R18" s="37"/>
+    <row r="18" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="21"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="47"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="36"/>
+      <c r="O18" s="35"/>
+      <c r="P18" s="35"/>
+      <c r="Q18" s="35"/>
+      <c r="R18" s="35"/>
       <c r="S18" s="5"/>
-      <c r="T18" s="37"/>
-      <c r="U18" s="37"/>
-      <c r="V18" s="37"/>
+      <c r="T18" s="35"/>
+      <c r="U18" s="35"/>
+      <c r="V18" s="35"/>
       <c r="W18" s="5"/>
-      <c r="X18" s="37"/>
-      <c r="Y18" s="37"/>
-      <c r="Z18" s="37"/>
-      <c r="AA18" s="30"/>
-      <c r="AB18" s="30"/>
-      <c r="AC18" s="30"/>
-      <c r="AD18" s="31"/>
-      <c r="AE18" s="31"/>
-      <c r="AF18" s="31"/>
-      <c r="AG18" s="31"/>
-      <c r="AH18" s="31"/>
-      <c r="AI18" s="31"/>
-      <c r="AJ18" s="31"/>
-      <c r="AK18" s="31"/>
-      <c r="AL18" s="31"/>
-      <c r="AM18" s="31"/>
+      <c r="X18" s="35"/>
+      <c r="Y18" s="35"/>
+      <c r="Z18" s="35"/>
+      <c r="AA18" s="28"/>
+      <c r="AB18" s="28"/>
+      <c r="AC18" s="28"/>
+      <c r="AD18" s="29"/>
+      <c r="AE18" s="29"/>
+      <c r="AF18" s="29"/>
+      <c r="AG18" s="29"/>
+      <c r="AH18" s="29"/>
+      <c r="AI18" s="29"/>
+      <c r="AJ18" s="29"/>
+      <c r="AK18" s="29"/>
+      <c r="AL18" s="29"/>
+      <c r="AM18" s="29"/>
     </row>
-    <row r="19" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="58"/>
-      <c r="I19" s="59"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="38"/>
-      <c r="O19" s="37"/>
-      <c r="P19" s="37"/>
-      <c r="Q19" s="37"/>
-      <c r="R19" s="37"/>
+    <row r="19" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="21"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="24"/>
+      <c r="L19" s="36"/>
+      <c r="O19" s="35"/>
+      <c r="P19" s="35"/>
+      <c r="Q19" s="35"/>
+      <c r="R19" s="35"/>
       <c r="S19" s="5"/>
-      <c r="T19" s="37"/>
-      <c r="U19" s="37"/>
-      <c r="V19" s="37"/>
+      <c r="T19" s="35"/>
+      <c r="U19" s="35"/>
+      <c r="V19" s="35"/>
       <c r="W19" s="5"/>
-      <c r="X19" s="37"/>
-      <c r="Y19" s="37"/>
-      <c r="Z19" s="37"/>
-      <c r="AA19" s="30"/>
-      <c r="AB19" s="30"/>
-      <c r="AC19" s="30"/>
-      <c r="AD19" s="31"/>
-      <c r="AE19" s="31"/>
-      <c r="AF19" s="31"/>
-      <c r="AG19" s="31"/>
-      <c r="AH19" s="31"/>
-      <c r="AI19" s="31"/>
-      <c r="AJ19" s="31"/>
-      <c r="AK19" s="31"/>
-      <c r="AL19" s="31"/>
-      <c r="AM19" s="31"/>
+      <c r="X19" s="35"/>
+      <c r="Y19" s="35"/>
+      <c r="Z19" s="35"/>
+      <c r="AA19" s="28"/>
+      <c r="AB19" s="28"/>
+      <c r="AC19" s="28"/>
+      <c r="AD19" s="29"/>
+      <c r="AE19" s="29"/>
+      <c r="AF19" s="29"/>
+      <c r="AG19" s="29"/>
+      <c r="AH19" s="29"/>
+      <c r="AI19" s="29"/>
+      <c r="AJ19" s="29"/>
+      <c r="AK19" s="29"/>
+      <c r="AL19" s="29"/>
+      <c r="AM19" s="29"/>
     </row>
-    <row r="20" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="23"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="58"/>
-      <c r="I20" s="59"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="38"/>
-      <c r="O20" s="37"/>
-      <c r="P20" s="37"/>
-      <c r="Q20" s="37"/>
-      <c r="R20" s="37"/>
+    <row r="20" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="21"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="36"/>
+      <c r="O20" s="35"/>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="35"/>
+      <c r="R20" s="35"/>
       <c r="S20" s="5"/>
-      <c r="T20" s="37"/>
-      <c r="U20" s="37"/>
-      <c r="V20" s="37"/>
+      <c r="T20" s="35"/>
+      <c r="U20" s="35"/>
+      <c r="V20" s="35"/>
       <c r="W20" s="5"/>
-      <c r="X20" s="37"/>
-      <c r="Y20" s="37"/>
-      <c r="Z20" s="37"/>
-      <c r="AA20" s="30"/>
-      <c r="AB20" s="30"/>
-      <c r="AC20" s="30"/>
-      <c r="AD20" s="31"/>
-      <c r="AE20" s="31"/>
-      <c r="AF20" s="31"/>
-      <c r="AG20" s="31"/>
-      <c r="AH20" s="31"/>
-      <c r="AI20" s="31"/>
-      <c r="AJ20" s="31"/>
-      <c r="AK20" s="31"/>
-      <c r="AL20" s="31"/>
-      <c r="AM20" s="31"/>
+      <c r="X20" s="35"/>
+      <c r="Y20" s="35"/>
+      <c r="Z20" s="35"/>
+      <c r="AA20" s="28"/>
+      <c r="AB20" s="28"/>
+      <c r="AC20" s="28"/>
+      <c r="AD20" s="29"/>
+      <c r="AE20" s="29"/>
+      <c r="AF20" s="29"/>
+      <c r="AG20" s="29"/>
+      <c r="AH20" s="29"/>
+      <c r="AI20" s="29"/>
+      <c r="AJ20" s="29"/>
+      <c r="AK20" s="29"/>
+      <c r="AL20" s="29"/>
+      <c r="AM20" s="29"/>
     </row>
-    <row r="21" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="23"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="58"/>
-      <c r="I21" s="59"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="38"/>
-      <c r="O21" s="37"/>
-      <c r="P21" s="37"/>
-      <c r="Q21" s="37"/>
-      <c r="R21" s="37"/>
+    <row r="21" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="21"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="45"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="47"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="36"/>
+      <c r="O21" s="35"/>
+      <c r="P21" s="35"/>
+      <c r="Q21" s="35"/>
+      <c r="R21" s="35"/>
       <c r="S21" s="5"/>
-      <c r="T21" s="37"/>
-      <c r="U21" s="37"/>
-      <c r="V21" s="37"/>
+      <c r="T21" s="35"/>
+      <c r="U21" s="35"/>
+      <c r="V21" s="35"/>
       <c r="W21" s="5"/>
-      <c r="X21" s="37"/>
-      <c r="Y21" s="37"/>
-      <c r="Z21" s="37"/>
-      <c r="AA21" s="30"/>
-      <c r="AB21" s="30"/>
-      <c r="AC21" s="30"/>
-      <c r="AD21" s="31"/>
-      <c r="AE21" s="31"/>
-      <c r="AF21" s="31"/>
-      <c r="AG21" s="31"/>
-      <c r="AH21" s="31"/>
-      <c r="AI21" s="31"/>
-      <c r="AJ21" s="31"/>
-      <c r="AK21" s="31"/>
-      <c r="AL21" s="31"/>
-      <c r="AM21" s="31"/>
+      <c r="X21" s="35"/>
+      <c r="Y21" s="35"/>
+      <c r="Z21" s="35"/>
+      <c r="AA21" s="28"/>
+      <c r="AB21" s="28"/>
+      <c r="AC21" s="28"/>
+      <c r="AD21" s="29"/>
+      <c r="AE21" s="29"/>
+      <c r="AF21" s="29"/>
+      <c r="AG21" s="29"/>
+      <c r="AH21" s="29"/>
+      <c r="AI21" s="29"/>
+      <c r="AJ21" s="29"/>
+      <c r="AK21" s="29"/>
+      <c r="AL21" s="29"/>
+      <c r="AM21" s="29"/>
     </row>
-    <row r="22" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="23"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="58"/>
-      <c r="I22" s="59"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="26"/>
-      <c r="L22" s="38"/>
-      <c r="O22" s="37"/>
-      <c r="P22" s="37"/>
-      <c r="Q22" s="37"/>
-      <c r="R22" s="37"/>
+    <row r="22" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="21"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="46"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="36"/>
+      <c r="O22" s="35"/>
+      <c r="P22" s="35"/>
+      <c r="Q22" s="35"/>
+      <c r="R22" s="35"/>
       <c r="S22" s="5"/>
-      <c r="T22" s="37"/>
-      <c r="U22" s="37"/>
-      <c r="V22" s="37"/>
+      <c r="T22" s="35"/>
+      <c r="U22" s="35"/>
+      <c r="V22" s="35"/>
       <c r="W22" s="5"/>
-      <c r="X22" s="37"/>
-      <c r="Y22" s="37"/>
-      <c r="Z22" s="37"/>
-      <c r="AA22" s="30"/>
-      <c r="AB22" s="30"/>
-      <c r="AC22" s="30"/>
-      <c r="AD22" s="31"/>
-      <c r="AE22" s="31"/>
-      <c r="AF22" s="31"/>
-      <c r="AG22" s="31"/>
-      <c r="AH22" s="31"/>
-      <c r="AI22" s="31"/>
-      <c r="AJ22" s="31"/>
-      <c r="AK22" s="31"/>
-      <c r="AL22" s="31"/>
-      <c r="AM22" s="31"/>
+      <c r="X22" s="35"/>
+      <c r="Y22" s="35"/>
+      <c r="Z22" s="35"/>
+      <c r="AA22" s="28"/>
+      <c r="AB22" s="28"/>
+      <c r="AC22" s="28"/>
+      <c r="AD22" s="29"/>
+      <c r="AE22" s="29"/>
+      <c r="AF22" s="29"/>
+      <c r="AG22" s="29"/>
+      <c r="AH22" s="29"/>
+      <c r="AI22" s="29"/>
+      <c r="AJ22" s="29"/>
+      <c r="AK22" s="29"/>
+      <c r="AL22" s="29"/>
+      <c r="AM22" s="29"/>
     </row>
-    <row r="23" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="23"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="58"/>
-      <c r="I23" s="59"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="26"/>
-      <c r="L23" s="38"/>
-      <c r="O23" s="37"/>
-      <c r="P23" s="37"/>
-      <c r="Q23" s="37"/>
-      <c r="R23" s="37"/>
+    <row r="23" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="21"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="36"/>
+      <c r="O23" s="35"/>
+      <c r="P23" s="35"/>
+      <c r="Q23" s="35"/>
+      <c r="R23" s="35"/>
       <c r="S23" s="5"/>
-      <c r="T23" s="37"/>
-      <c r="U23" s="37"/>
-      <c r="V23" s="37"/>
+      <c r="T23" s="35"/>
+      <c r="U23" s="35"/>
+      <c r="V23" s="35"/>
       <c r="W23" s="5"/>
-      <c r="X23" s="37"/>
-      <c r="Y23" s="37"/>
-      <c r="Z23" s="37"/>
-      <c r="AA23" s="30"/>
-      <c r="AB23" s="30"/>
-      <c r="AC23" s="30"/>
-      <c r="AD23" s="31"/>
-      <c r="AE23" s="31"/>
-      <c r="AF23" s="31"/>
-      <c r="AG23" s="31"/>
-      <c r="AH23" s="31"/>
-      <c r="AI23" s="31"/>
-      <c r="AJ23" s="31"/>
-      <c r="AK23" s="31"/>
-      <c r="AL23" s="31"/>
-      <c r="AM23" s="31"/>
+      <c r="X23" s="35"/>
+      <c r="Y23" s="35"/>
+      <c r="Z23" s="35"/>
+      <c r="AA23" s="28"/>
+      <c r="AB23" s="28"/>
+      <c r="AC23" s="28"/>
+      <c r="AD23" s="29"/>
+      <c r="AE23" s="29"/>
+      <c r="AF23" s="29"/>
+      <c r="AG23" s="29"/>
+      <c r="AH23" s="29"/>
+      <c r="AI23" s="29"/>
+      <c r="AJ23" s="29"/>
+      <c r="AK23" s="29"/>
+      <c r="AL23" s="29"/>
+      <c r="AM23" s="29"/>
     </row>
-    <row r="24" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="23"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="59"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="26"/>
-      <c r="L24" s="38"/>
-      <c r="O24" s="37"/>
-      <c r="P24" s="37"/>
-      <c r="Q24" s="37"/>
-      <c r="R24" s="37"/>
+    <row r="24" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="21"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="47"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="36"/>
+      <c r="O24" s="35"/>
+      <c r="P24" s="35"/>
+      <c r="Q24" s="35"/>
+      <c r="R24" s="35"/>
       <c r="S24" s="5"/>
-      <c r="T24" s="37"/>
-      <c r="U24" s="37"/>
-      <c r="V24" s="37"/>
+      <c r="T24" s="35"/>
+      <c r="U24" s="35"/>
+      <c r="V24" s="35"/>
       <c r="W24" s="5"/>
-      <c r="X24" s="37"/>
-      <c r="Y24" s="37"/>
-      <c r="Z24" s="37"/>
-      <c r="AA24" s="30"/>
-      <c r="AB24" s="30"/>
-      <c r="AC24" s="30"/>
-      <c r="AD24" s="31"/>
-      <c r="AE24" s="31"/>
-      <c r="AF24" s="31"/>
-      <c r="AG24" s="31"/>
-      <c r="AH24" s="31"/>
-      <c r="AI24" s="31"/>
-      <c r="AJ24" s="31"/>
-      <c r="AK24" s="31"/>
-      <c r="AL24" s="31"/>
-      <c r="AM24" s="31"/>
+      <c r="X24" s="35"/>
+      <c r="Y24" s="35"/>
+      <c r="Z24" s="35"/>
+      <c r="AA24" s="28"/>
+      <c r="AB24" s="28"/>
+      <c r="AC24" s="28"/>
+      <c r="AD24" s="29"/>
+      <c r="AE24" s="29"/>
+      <c r="AF24" s="29"/>
+      <c r="AG24" s="29"/>
+      <c r="AH24" s="29"/>
+      <c r="AI24" s="29"/>
+      <c r="AJ24" s="29"/>
+      <c r="AK24" s="29"/>
+      <c r="AL24" s="29"/>
+      <c r="AM24" s="29"/>
     </row>
-    <row r="25" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="58"/>
-      <c r="I25" s="59"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="38"/>
-      <c r="O25" s="37"/>
-      <c r="P25" s="37"/>
-      <c r="Q25" s="37"/>
-      <c r="R25" s="37"/>
+    <row r="25" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="47"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="36"/>
+      <c r="O25" s="35"/>
+      <c r="P25" s="35"/>
+      <c r="Q25" s="35"/>
+      <c r="R25" s="35"/>
       <c r="S25" s="5"/>
-      <c r="T25" s="37"/>
-      <c r="U25" s="37"/>
-      <c r="V25" s="37"/>
+      <c r="T25" s="35"/>
+      <c r="U25" s="35"/>
+      <c r="V25" s="35"/>
       <c r="W25" s="5"/>
-      <c r="X25" s="37"/>
-      <c r="Y25" s="37"/>
-      <c r="Z25" s="37"/>
-      <c r="AA25" s="30"/>
-      <c r="AB25" s="30"/>
-      <c r="AC25" s="30"/>
-      <c r="AD25" s="31"/>
-      <c r="AE25" s="31"/>
-      <c r="AF25" s="31"/>
-      <c r="AG25" s="31"/>
-      <c r="AH25" s="31"/>
-      <c r="AI25" s="31"/>
-      <c r="AJ25" s="31"/>
-      <c r="AK25" s="31"/>
-      <c r="AL25" s="31"/>
-      <c r="AM25" s="31"/>
+      <c r="X25" s="35"/>
+      <c r="Y25" s="35"/>
+      <c r="Z25" s="35"/>
+      <c r="AA25" s="28"/>
+      <c r="AB25" s="28"/>
+      <c r="AC25" s="28"/>
+      <c r="AD25" s="29"/>
+      <c r="AE25" s="29"/>
+      <c r="AF25" s="29"/>
+      <c r="AG25" s="29"/>
+      <c r="AH25" s="29"/>
+      <c r="AI25" s="29"/>
+      <c r="AJ25" s="29"/>
+      <c r="AK25" s="29"/>
+      <c r="AL25" s="29"/>
+      <c r="AM25" s="29"/>
     </row>
-    <row r="26" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="23"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="38"/>
-      <c r="O26" s="37"/>
-      <c r="P26" s="37"/>
-      <c r="Q26" s="37"/>
-      <c r="R26" s="37"/>
+    <row r="26" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="21"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="46"/>
+      <c r="I26" s="47"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="36"/>
+      <c r="O26" s="35"/>
+      <c r="P26" s="35"/>
+      <c r="Q26" s="35"/>
+      <c r="R26" s="35"/>
       <c r="S26" s="5"/>
-      <c r="T26" s="37"/>
-      <c r="U26" s="37"/>
-      <c r="V26" s="37"/>
+      <c r="T26" s="35"/>
+      <c r="U26" s="35"/>
+      <c r="V26" s="35"/>
       <c r="W26" s="5"/>
-      <c r="X26" s="37"/>
-      <c r="Y26" s="37"/>
-      <c r="Z26" s="37"/>
-      <c r="AA26" s="30"/>
-      <c r="AB26" s="30"/>
-      <c r="AC26" s="30"/>
-      <c r="AD26" s="31"/>
-      <c r="AE26" s="31"/>
-      <c r="AF26" s="31"/>
-      <c r="AG26" s="31"/>
-      <c r="AH26" s="31"/>
-      <c r="AI26" s="31"/>
-      <c r="AJ26" s="31"/>
-      <c r="AK26" s="31"/>
-      <c r="AL26" s="31"/>
-      <c r="AM26" s="31"/>
+      <c r="X26" s="35"/>
+      <c r="Y26" s="35"/>
+      <c r="Z26" s="35"/>
+      <c r="AA26" s="28"/>
+      <c r="AB26" s="28"/>
+      <c r="AC26" s="28"/>
+      <c r="AD26" s="29"/>
+      <c r="AE26" s="29"/>
+      <c r="AF26" s="29"/>
+      <c r="AG26" s="29"/>
+      <c r="AH26" s="29"/>
+      <c r="AI26" s="29"/>
+      <c r="AJ26" s="29"/>
+      <c r="AK26" s="29"/>
+      <c r="AL26" s="29"/>
+      <c r="AM26" s="29"/>
     </row>
-    <row r="27" spans="2:39" s="29" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="23"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="58"/>
-      <c r="I27" s="59"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="38"/>
-      <c r="O27" s="37"/>
-      <c r="P27" s="37"/>
-      <c r="Q27" s="37"/>
-      <c r="R27" s="37"/>
+    <row r="27" spans="2:39" s="27" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="21"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="47"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="36"/>
+      <c r="O27" s="35"/>
+      <c r="P27" s="35"/>
+      <c r="Q27" s="35"/>
+      <c r="R27" s="35"/>
       <c r="S27" s="5"/>
-      <c r="T27" s="37"/>
-      <c r="U27" s="37"/>
-      <c r="V27" s="37"/>
+      <c r="T27" s="35"/>
+      <c r="U27" s="35"/>
+      <c r="V27" s="35"/>
       <c r="W27" s="5"/>
-      <c r="X27" s="37"/>
-      <c r="Y27" s="37"/>
-      <c r="Z27" s="37"/>
-      <c r="AA27" s="30"/>
-      <c r="AB27" s="30"/>
-      <c r="AC27" s="30"/>
-      <c r="AD27" s="31"/>
-      <c r="AE27" s="31"/>
-      <c r="AF27" s="31"/>
-      <c r="AG27" s="31"/>
-      <c r="AH27" s="31"/>
-      <c r="AI27" s="31"/>
-      <c r="AJ27" s="31"/>
-      <c r="AK27" s="31"/>
-      <c r="AL27" s="31"/>
-      <c r="AM27" s="31"/>
+      <c r="X27" s="35"/>
+      <c r="Y27" s="35"/>
+      <c r="Z27" s="35"/>
+      <c r="AA27" s="28"/>
+      <c r="AB27" s="28"/>
+      <c r="AC27" s="28"/>
+      <c r="AD27" s="29"/>
+      <c r="AE27" s="29"/>
+      <c r="AF27" s="29"/>
+      <c r="AG27" s="29"/>
+      <c r="AH27" s="29"/>
+      <c r="AI27" s="29"/>
+      <c r="AJ27" s="29"/>
+      <c r="AK27" s="29"/>
+      <c r="AL27" s="29"/>
+      <c r="AM27" s="29"/>
     </row>
     <row r="28" spans="2:39" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="44" t="s">
+      <c r="B28" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="45"/>
-      <c r="H28" s="45"/>
-      <c r="I28" s="45"/>
-      <c r="J28" s="46"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="63"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="63"/>
+      <c r="I28" s="63"/>
+      <c r="J28" s="75"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
       <c r="O28" s="6"/>
       <c r="P28" s="6"/>
       <c r="Q28" s="6"/>
@@ -3498,19 +3434,19 @@
       <c r="AM28" s="4"/>
     </row>
     <row r="29" spans="2:39" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="44" t="s">
-        <v>24</v>
+      <c r="B29" s="64" t="s">
+        <v>25</v>
       </c>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="45"/>
-      <c r="J29" s="46"/>
-      <c r="K29" s="22"/>
-      <c r="L29" s="22"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
+      <c r="E29" s="63"/>
+      <c r="F29" s="63"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="63"/>
+      <c r="I29" s="63"/>
+      <c r="J29" s="75"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="20"/>
       <c r="N29" s="10"/>
       <c r="O29" s="9"/>
       <c r="P29" s="9"/>
@@ -3538,108 +3474,122 @@
       <c r="AL29" s="4"/>
       <c r="AM29" s="4"/>
     </row>
-    <row r="30" spans="2:39" s="1" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="66" t="s">
+    <row r="30" spans="2:39" s="65" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B30" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" s="63"/>
+      <c r="D30" s="63"/>
+      <c r="E30" s="63"/>
+      <c r="F30" s="63"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="63"/>
+      <c r="I30" s="63"/>
+      <c r="J30" s="75"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="20"/>
+      <c r="N30" s="72"/>
+      <c r="O30" s="71"/>
+      <c r="P30" s="71"/>
+      <c r="Q30" s="71"/>
+      <c r="R30" s="71"/>
+      <c r="S30" s="70"/>
+      <c r="T30" s="71"/>
+      <c r="U30" s="71"/>
+      <c r="V30" s="71"/>
+      <c r="W30" s="67"/>
+      <c r="X30" s="69"/>
+      <c r="Y30" s="69"/>
+      <c r="Z30" s="69"/>
+      <c r="AA30" s="68"/>
+      <c r="AB30" s="68"/>
+      <c r="AC30" s="68"/>
+      <c r="AD30" s="68"/>
+      <c r="AE30" s="68"/>
+      <c r="AF30" s="68"/>
+      <c r="AG30" s="68"/>
+      <c r="AH30" s="68"/>
+      <c r="AI30" s="68"/>
+      <c r="AJ30" s="68"/>
+      <c r="AK30" s="68"/>
+      <c r="AL30" s="68"/>
+      <c r="AM30" s="68"/>
+    </row>
+    <row r="31" spans="2:39" s="65" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="60"/>
-      <c r="D30" s="61"/>
-      <c r="E30" s="61"/>
-      <c r="F30" s="61"/>
-      <c r="G30" s="61"/>
-      <c r="H30" s="61"/>
-      <c r="I30" s="61"/>
-      <c r="J30" s="61"/>
-      <c r="K30" s="61"/>
-      <c r="L30" s="62"/>
-      <c r="N30" s="11"/>
-      <c r="O30" s="12"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="2"/>
-      <c r="Y30" s="2"/>
-      <c r="Z30" s="2"/>
-      <c r="AA30" s="4"/>
-      <c r="AB30" s="4"/>
-      <c r="AC30" s="4"/>
-      <c r="AD30" s="4"/>
-      <c r="AE30" s="4"/>
-      <c r="AF30" s="4"/>
-      <c r="AG30" s="4"/>
-      <c r="AH30" s="4"/>
-      <c r="AI30" s="4"/>
-      <c r="AJ30" s="4"/>
-      <c r="AK30" s="4"/>
-      <c r="AL30" s="4"/>
-      <c r="AM30" s="4"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
+      <c r="J31" s="38"/>
+      <c r="K31" s="38"/>
+      <c r="L31" s="39"/>
+      <c r="N31" s="73"/>
+      <c r="O31" s="74"/>
+      <c r="P31" s="66"/>
+      <c r="Q31" s="66"/>
+      <c r="R31" s="66"/>
+      <c r="S31" s="66"/>
+      <c r="T31" s="66"/>
+      <c r="U31" s="66"/>
+      <c r="V31" s="66"/>
+      <c r="W31" s="66"/>
+      <c r="X31" s="66"/>
+      <c r="Y31" s="66"/>
+      <c r="Z31" s="66"/>
+      <c r="AA31" s="68"/>
+      <c r="AB31" s="68"/>
+      <c r="AC31" s="68"/>
+      <c r="AD31" s="68"/>
+      <c r="AE31" s="68"/>
+      <c r="AF31" s="68"/>
+      <c r="AG31" s="68"/>
+      <c r="AH31" s="68"/>
+      <c r="AI31" s="68"/>
+      <c r="AJ31" s="68"/>
+      <c r="AK31" s="68"/>
+      <c r="AL31" s="68"/>
+      <c r="AM31" s="68"/>
     </row>
-    <row r="31" spans="2:39" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="67"/>
-      <c r="C31" s="63"/>
-      <c r="D31" s="64"/>
-      <c r="E31" s="64"/>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
-      <c r="H31" s="64"/>
-      <c r="I31" s="64"/>
-      <c r="J31" s="64"/>
-      <c r="K31" s="64"/>
-      <c r="L31" s="65"/>
-      <c r="O31" s="2"/>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="2"/>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="2"/>
-      <c r="W31" s="2"/>
-      <c r="X31" s="2"/>
-      <c r="Y31" s="2"/>
-      <c r="Z31" s="2"/>
-      <c r="AA31" s="4"/>
-      <c r="AB31" s="4"/>
-      <c r="AC31" s="4"/>
-      <c r="AD31" s="4"/>
-      <c r="AE31" s="4"/>
-      <c r="AF31" s="4"/>
-      <c r="AG31" s="4"/>
-      <c r="AH31" s="4"/>
-      <c r="AI31" s="4"/>
-      <c r="AJ31" s="4"/>
-      <c r="AK31" s="4"/>
-      <c r="AL31" s="4"/>
-      <c r="AM31" s="4"/>
+    <row r="32" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="B32" s="44"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="41"/>
+      <c r="K32" s="41"/>
+      <c r="L32" s="42"/>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange password="C71F" sqref="O11:Z29" name="Aralık1_1"/>
+    <protectedRange password="C71F" sqref="O11:Z30" name="Aralık1_1"/>
   </protectedRanges>
-  <mergeCells count="51">
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:H10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="I9:J9"/>
+  <mergeCells count="50">
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="B28:J28"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="X12:Z12"/>
@@ -3656,186 +3606,187 @@
     <mergeCell ref="E8:H8"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="K8:L8"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:L31"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="B28:J28"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G18:I18"/>
   </mergeCells>
   <conditionalFormatting sqref="J12:K12 K16">
-    <cfRule type="cellIs" dxfId="152" priority="247" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="248" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="249" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="247" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="142" priority="248" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="141" priority="249" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="cellIs" dxfId="146" priority="178" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="179" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="180" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="178" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="139" priority="179" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="180" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6">
-    <cfRule type="cellIs" dxfId="143" priority="172" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="173" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="174" operator="equal">
+    <cfRule type="cellIs" dxfId="137" priority="172" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="173" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="135" priority="174" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7">
-    <cfRule type="cellIs" dxfId="140" priority="160" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="161" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="162" operator="equal">
+    <cfRule type="cellIs" dxfId="134" priority="160" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="161" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="162" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K15">
-    <cfRule type="cellIs" dxfId="134" priority="145" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="146" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="147" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="145" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="146" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="129" priority="147" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="cellIs" dxfId="131" priority="142" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="143" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="144" operator="equal">
+    <cfRule type="cellIs" dxfId="128" priority="142" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="127" priority="143" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="126" priority="144" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K14">
-    <cfRule type="cellIs" dxfId="128" priority="139" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="140" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="141" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="139" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="140" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="141" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="cellIs" dxfId="125" priority="136" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="137" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="138" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="136" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="121" priority="137" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="138" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K13">
-    <cfRule type="cellIs" dxfId="122" priority="133" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="134" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="135" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="133" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="134" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="117" priority="135" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J13">
-    <cfRule type="cellIs" dxfId="119" priority="130" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="131" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="132" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="130" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="131" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="114" priority="132" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="cellIs" dxfId="116" priority="127" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="128" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="129" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="127" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="112" priority="128" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="129" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
-    <cfRule type="cellIs" dxfId="113" priority="124" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="125" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="126" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="124" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="125" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="108" priority="126" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K8">
-    <cfRule type="cellIs" dxfId="110" priority="121" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="122" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="123" operator="equal">
+    <cfRule type="cellIs" dxfId="107" priority="121" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="122" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="123" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K17">
-    <cfRule type="cellIs" dxfId="107" priority="109" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="110" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="111" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="109" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="110" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="111" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="cellIs" dxfId="104" priority="103" operator="equal">
-      <formula>"h"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="104" operator="equal">
-      <formula>"k"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="105" operator="equal">
+    <cfRule type="cellIs" dxfId="101" priority="103" operator="equal">
+      <formula>"h"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="104" operator="equal">
+      <formula>"k"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="99" priority="105" operator="equal">
       <formula>"e"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
dğzeltme: taslakların yıl gün ay satırları düzeltildi
</commit_message>
<xml_diff>
--- a/docs/cikti_taslagi.xlsx
+++ b/docs/cikti_taslagi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammed.bulut\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641C9AEA-0D55-4354-B71B-FE0CF98FAFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A58105F1-6DC2-4E18-AEE8-CF965E03BCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -574,66 +574,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -660,8 +600,68 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2484,13 +2484,13 @@
       <c r="G2" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="53" t="s">
+      <c r="H2" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="55"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="69"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
@@ -2511,11 +2511,11 @@
       <c r="E3" s="17"/>
       <c r="F3" s="33"/>
       <c r="G3" s="34"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57"/>
-      <c r="L3" s="58"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="72"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -2530,19 +2530,19 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="2:39" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -2561,24 +2561,24 @@
     </row>
     <row r="5" spans="2:39" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="15"/>
-      <c r="C5" s="60" t="s">
+      <c r="C5" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60" t="s">
+      <c r="D5" s="58"/>
+      <c r="E5" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
-      <c r="I5" s="60" t="s">
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="J5" s="60"/>
-      <c r="K5" s="60" t="s">
+      <c r="J5" s="58"/>
+      <c r="K5" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="60"/>
+      <c r="L5" s="58"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -2597,16 +2597,16 @@
     </row>
     <row r="6" spans="2:39" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="18"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="61"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="49"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
       <c r="O6" s="11"/>
       <c r="P6" s="11"/>
       <c r="Q6" s="11"/>
@@ -2625,16 +2625,16 @@
     </row>
     <row r="7" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="18"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="51"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="61"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="59"/>
+      <c r="L7" s="59"/>
       <c r="O7" s="11"/>
       <c r="P7" s="11"/>
       <c r="Q7" s="11"/>
@@ -2653,16 +2653,16 @@
     </row>
     <row r="8" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="18"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="49"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="49"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="51"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="48"/>
-      <c r="L8" s="48"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="62"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="75"/>
       <c r="O8" s="11"/>
       <c r="P8" s="11"/>
       <c r="Q8" s="11"/>
@@ -2681,16 +2681,16 @@
     </row>
     <row r="9" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="18"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="51"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="48"/>
-      <c r="L9" s="48"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="75"/>
       <c r="O9" s="11"/>
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
@@ -2709,16 +2709,16 @@
     </row>
     <row r="10" spans="2:39" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="18"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="51"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="48"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="75"/>
+      <c r="L10" s="75"/>
       <c r="O10" s="11"/>
       <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
@@ -2736,21 +2736,21 @@
       <c r="AC10" s="2"/>
     </row>
     <row r="11" spans="2:39" s="1" customFormat="1" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="60" t="s">
+      <c r="B11" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60" t="s">
+      <c r="C11" s="58"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
+      <c r="H11" s="58"/>
+      <c r="I11" s="58"/>
+      <c r="J11" s="58"/>
+      <c r="K11" s="58"/>
+      <c r="L11" s="58"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
@@ -2783,11 +2783,11 @@
       <c r="F12" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="62" t="s">
+      <c r="G12" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
+      <c r="H12" s="66"/>
+      <c r="I12" s="66"/>
       <c r="J12" s="12" t="s">
         <v>12</v>
       </c>
@@ -2797,18 +2797,18 @@
       <c r="L12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="O12" s="59"/>
-      <c r="P12" s="59"/>
-      <c r="Q12" s="59"/>
+      <c r="O12" s="73"/>
+      <c r="P12" s="73"/>
+      <c r="Q12" s="73"/>
       <c r="R12" s="35"/>
       <c r="S12" s="5"/>
-      <c r="T12" s="59"/>
-      <c r="U12" s="59"/>
-      <c r="V12" s="59"/>
+      <c r="T12" s="73"/>
+      <c r="U12" s="73"/>
+      <c r="V12" s="73"/>
       <c r="W12" s="5"/>
-      <c r="X12" s="59"/>
-      <c r="Y12" s="59"/>
-      <c r="Z12" s="59"/>
+      <c r="X12" s="73"/>
+      <c r="Y12" s="73"/>
+      <c r="Z12" s="73"/>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
       <c r="AC12" s="2"/>
@@ -2829,9 +2829,9 @@
       <c r="D13" s="22"/>
       <c r="E13" s="23"/>
       <c r="F13" s="23"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="46"/>
-      <c r="I13" s="47"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="64"/>
+      <c r="I13" s="65"/>
       <c r="J13" s="14"/>
       <c r="K13" s="24"/>
       <c r="L13" s="36"/>
@@ -2867,9 +2867,9 @@
       <c r="D14" s="22"/>
       <c r="E14" s="23"/>
       <c r="F14" s="23"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="47"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="65"/>
       <c r="J14" s="14"/>
       <c r="K14" s="24"/>
       <c r="L14" s="36"/>
@@ -2905,9 +2905,9 @@
       <c r="D15" s="22"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="47"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="65"/>
       <c r="J15" s="14"/>
       <c r="K15" s="24"/>
       <c r="L15" s="36"/>
@@ -2943,9 +2943,9 @@
       <c r="D16" s="22"/>
       <c r="E16" s="23"/>
       <c r="F16" s="23"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="47"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="64"/>
+      <c r="I16" s="65"/>
       <c r="J16" s="14"/>
       <c r="K16" s="24"/>
       <c r="L16" s="36"/>
@@ -2981,9 +2981,9 @@
       <c r="D17" s="22"/>
       <c r="E17" s="23"/>
       <c r="F17" s="23"/>
-      <c r="G17" s="45"/>
-      <c r="H17" s="46"/>
-      <c r="I17" s="47"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="64"/>
+      <c r="I17" s="65"/>
       <c r="J17" s="14"/>
       <c r="K17" s="24"/>
       <c r="L17" s="36"/>
@@ -3019,9 +3019,9 @@
       <c r="D18" s="22"/>
       <c r="E18" s="23"/>
       <c r="F18" s="23"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="47"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="64"/>
+      <c r="I18" s="65"/>
       <c r="J18" s="14"/>
       <c r="K18" s="24"/>
       <c r="L18" s="36"/>
@@ -3057,9 +3057,9 @@
       <c r="D19" s="22"/>
       <c r="E19" s="23"/>
       <c r="F19" s="23"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="46"/>
-      <c r="I19" s="47"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="64"/>
+      <c r="I19" s="65"/>
       <c r="J19" s="14"/>
       <c r="K19" s="24"/>
       <c r="L19" s="36"/>
@@ -3095,9 +3095,9 @@
       <c r="D20" s="22"/>
       <c r="E20" s="23"/>
       <c r="F20" s="23"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="47"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="64"/>
+      <c r="I20" s="65"/>
       <c r="J20" s="14"/>
       <c r="K20" s="24"/>
       <c r="L20" s="36"/>
@@ -3133,9 +3133,9 @@
       <c r="D21" s="22"/>
       <c r="E21" s="23"/>
       <c r="F21" s="23"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="46"/>
-      <c r="I21" s="47"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="64"/>
+      <c r="I21" s="65"/>
       <c r="J21" s="14"/>
       <c r="K21" s="24"/>
       <c r="L21" s="36"/>
@@ -3171,9 +3171,9 @@
       <c r="D22" s="22"/>
       <c r="E22" s="23"/>
       <c r="F22" s="23"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="47"/>
+      <c r="G22" s="63"/>
+      <c r="H22" s="64"/>
+      <c r="I22" s="65"/>
       <c r="J22" s="14"/>
       <c r="K22" s="24"/>
       <c r="L22" s="36"/>
@@ -3209,9 +3209,9 @@
       <c r="D23" s="22"/>
       <c r="E23" s="23"/>
       <c r="F23" s="23"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="47"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="64"/>
+      <c r="I23" s="65"/>
       <c r="J23" s="14"/>
       <c r="K23" s="24"/>
       <c r="L23" s="36"/>
@@ -3247,9 +3247,9 @@
       <c r="D24" s="22"/>
       <c r="E24" s="23"/>
       <c r="F24" s="23"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="47"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="64"/>
+      <c r="I24" s="65"/>
       <c r="J24" s="14"/>
       <c r="K24" s="24"/>
       <c r="L24" s="36"/>
@@ -3285,9 +3285,9 @@
       <c r="D25" s="22"/>
       <c r="E25" s="23"/>
       <c r="F25" s="23"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="47"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="64"/>
+      <c r="I25" s="65"/>
       <c r="J25" s="14"/>
       <c r="K25" s="24"/>
       <c r="L25" s="36"/>
@@ -3323,9 +3323,9 @@
       <c r="D26" s="22"/>
       <c r="E26" s="23"/>
       <c r="F26" s="23"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="46"/>
-      <c r="I26" s="47"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="64"/>
+      <c r="I26" s="65"/>
       <c r="J26" s="14"/>
       <c r="K26" s="24"/>
       <c r="L26" s="36"/>
@@ -3361,9 +3361,9 @@
       <c r="D27" s="22"/>
       <c r="E27" s="23"/>
       <c r="F27" s="23"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="46"/>
-      <c r="I27" s="47"/>
+      <c r="G27" s="63"/>
+      <c r="H27" s="64"/>
+      <c r="I27" s="65"/>
       <c r="J27" s="14"/>
       <c r="K27" s="24"/>
       <c r="L27" s="36"/>
@@ -3394,17 +3394,17 @@
       <c r="AM27" s="29"/>
     </row>
     <row r="28" spans="2:39" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="64" t="s">
+      <c r="B28" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="63"/>
-      <c r="D28" s="63"/>
-      <c r="E28" s="63"/>
-      <c r="F28" s="63"/>
-      <c r="G28" s="63"/>
-      <c r="H28" s="63"/>
-      <c r="I28" s="63"/>
-      <c r="J28" s="75"/>
+      <c r="C28" s="56"/>
+      <c r="D28" s="56"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="56"/>
+      <c r="G28" s="56"/>
+      <c r="H28" s="56"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="57"/>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
       <c r="O28" s="6"/>
@@ -3434,17 +3434,17 @@
       <c r="AM28" s="4"/>
     </row>
     <row r="29" spans="2:39" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="64" t="s">
+      <c r="B29" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="C29" s="63"/>
-      <c r="D29" s="63"/>
-      <c r="E29" s="63"/>
-      <c r="F29" s="63"/>
-      <c r="G29" s="63"/>
-      <c r="H29" s="63"/>
-      <c r="I29" s="63"/>
-      <c r="J29" s="75"/>
+      <c r="C29" s="56"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="20"/>
       <c r="K29" s="20"/>
       <c r="L29" s="20"/>
       <c r="N29" s="10"/>
@@ -3474,48 +3474,48 @@
       <c r="AL29" s="4"/>
       <c r="AM29" s="4"/>
     </row>
-    <row r="30" spans="2:39" s="65" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B30" s="64" t="s">
+    <row r="30" spans="2:39" s="45" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B30" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="63"/>
-      <c r="D30" s="63"/>
-      <c r="E30" s="63"/>
-      <c r="F30" s="63"/>
-      <c r="G30" s="63"/>
-      <c r="H30" s="63"/>
-      <c r="I30" s="63"/>
-      <c r="J30" s="75"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="57"/>
       <c r="K30" s="20"/>
       <c r="L30" s="20"/>
-      <c r="N30" s="72"/>
-      <c r="O30" s="71"/>
-      <c r="P30" s="71"/>
-      <c r="Q30" s="71"/>
-      <c r="R30" s="71"/>
-      <c r="S30" s="70"/>
-      <c r="T30" s="71"/>
-      <c r="U30" s="71"/>
-      <c r="V30" s="71"/>
-      <c r="W30" s="67"/>
-      <c r="X30" s="69"/>
-      <c r="Y30" s="69"/>
-      <c r="Z30" s="69"/>
-      <c r="AA30" s="68"/>
-      <c r="AB30" s="68"/>
-      <c r="AC30" s="68"/>
-      <c r="AD30" s="68"/>
-      <c r="AE30" s="68"/>
-      <c r="AF30" s="68"/>
-      <c r="AG30" s="68"/>
-      <c r="AH30" s="68"/>
-      <c r="AI30" s="68"/>
-      <c r="AJ30" s="68"/>
-      <c r="AK30" s="68"/>
-      <c r="AL30" s="68"/>
-      <c r="AM30" s="68"/>
+      <c r="N30" s="52"/>
+      <c r="O30" s="51"/>
+      <c r="P30" s="51"/>
+      <c r="Q30" s="51"/>
+      <c r="R30" s="51"/>
+      <c r="S30" s="50"/>
+      <c r="T30" s="51"/>
+      <c r="U30" s="51"/>
+      <c r="V30" s="51"/>
+      <c r="W30" s="47"/>
+      <c r="X30" s="49"/>
+      <c r="Y30" s="49"/>
+      <c r="Z30" s="49"/>
+      <c r="AA30" s="48"/>
+      <c r="AB30" s="48"/>
+      <c r="AC30" s="48"/>
+      <c r="AD30" s="48"/>
+      <c r="AE30" s="48"/>
+      <c r="AF30" s="48"/>
+      <c r="AG30" s="48"/>
+      <c r="AH30" s="48"/>
+      <c r="AI30" s="48"/>
+      <c r="AJ30" s="48"/>
+      <c r="AK30" s="48"/>
+      <c r="AL30" s="48"/>
+      <c r="AM30" s="48"/>
     </row>
-    <row r="31" spans="2:39" s="65" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:39" s="45" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="43" t="s">
         <v>10</v>
       </c>
@@ -3529,32 +3529,32 @@
       <c r="J31" s="38"/>
       <c r="K31" s="38"/>
       <c r="L31" s="39"/>
-      <c r="N31" s="73"/>
-      <c r="O31" s="74"/>
-      <c r="P31" s="66"/>
-      <c r="Q31" s="66"/>
-      <c r="R31" s="66"/>
-      <c r="S31" s="66"/>
-      <c r="T31" s="66"/>
-      <c r="U31" s="66"/>
-      <c r="V31" s="66"/>
-      <c r="W31" s="66"/>
-      <c r="X31" s="66"/>
-      <c r="Y31" s="66"/>
-      <c r="Z31" s="66"/>
-      <c r="AA31" s="68"/>
-      <c r="AB31" s="68"/>
-      <c r="AC31" s="68"/>
-      <c r="AD31" s="68"/>
-      <c r="AE31" s="68"/>
-      <c r="AF31" s="68"/>
-      <c r="AG31" s="68"/>
-      <c r="AH31" s="68"/>
-      <c r="AI31" s="68"/>
-      <c r="AJ31" s="68"/>
-      <c r="AK31" s="68"/>
-      <c r="AL31" s="68"/>
-      <c r="AM31" s="68"/>
+      <c r="N31" s="53"/>
+      <c r="O31" s="54"/>
+      <c r="P31" s="46"/>
+      <c r="Q31" s="46"/>
+      <c r="R31" s="46"/>
+      <c r="S31" s="46"/>
+      <c r="T31" s="46"/>
+      <c r="U31" s="46"/>
+      <c r="V31" s="46"/>
+      <c r="W31" s="46"/>
+      <c r="X31" s="46"/>
+      <c r="Y31" s="46"/>
+      <c r="Z31" s="46"/>
+      <c r="AA31" s="48"/>
+      <c r="AB31" s="48"/>
+      <c r="AC31" s="48"/>
+      <c r="AD31" s="48"/>
+      <c r="AE31" s="48"/>
+      <c r="AF31" s="48"/>
+      <c r="AG31" s="48"/>
+      <c r="AH31" s="48"/>
+      <c r="AI31" s="48"/>
+      <c r="AJ31" s="48"/>
+      <c r="AK31" s="48"/>
+      <c r="AL31" s="48"/>
+      <c r="AM31" s="48"/>
     </row>
     <row r="32" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B32" s="44"/>
@@ -3574,22 +3574,10 @@
     <protectedRange password="C71F" sqref="O11:Z30" name="Aralık1_1"/>
   </protectedRanges>
   <mergeCells count="50">
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="B29:I29"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="X12:Z12"/>
@@ -3606,6 +3594,13 @@
     <mergeCell ref="E8:H8"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="K8:L8"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G12:I12"/>
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="E10:H10"/>
@@ -3614,6 +3609,14 @@
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="E9:H9"/>
     <mergeCell ref="I9:J9"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="B28:J28"/>
     <mergeCell ref="G27:I27"/>
     <mergeCell ref="G26:I26"/>
     <mergeCell ref="G25:I25"/>
@@ -3621,9 +3624,6 @@
     <mergeCell ref="G23:I23"/>
     <mergeCell ref="G22:I22"/>
     <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G18:I18"/>
   </mergeCells>
   <conditionalFormatting sqref="J12:K12 K16">
     <cfRule type="cellIs" dxfId="143" priority="247" operator="equal">

</xml_diff>